<commit_message>
Fill país de origen and integración nacional on sheet 1 for all 71 items
Co-authored-by: Miguel Angel Cruz Ortiz <Ylika.dev@outlook.com>
</commit_message>
<xml_diff>
--- a/ANEXO TECNICO POLICIA BANCARIA.xlsx
+++ b/ANEXO TECNICO POLICIA BANCARIA.xlsx
@@ -944,8 +944,14 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="n"/>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>CHINA</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G2" s="46" t="n"/>
       <c r="H2" s="1" t="n"/>
       <c r="I2" s="8" t="n"/>
@@ -980,8 +986,14 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E3" s="1" t="n"/>
-      <c r="F3" s="1" t="n"/>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>CHINA</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G3" s="46" t="n"/>
       <c r="H3" s="1" t="n"/>
       <c r="I3" s="8" t="n"/>
@@ -1016,9 +1028,19 @@
           <t>ROLLO</t>
         </is>
       </c>
-      <c r="E4" s="1" t="n"/>
-      <c r="F4" s="1" t="n"/>
-      <c r="G4" s="46" t="n"/>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G4" s="46" t="inlineStr">
+        <is>
+          <t>CONDUMEX</t>
+        </is>
+      </c>
       <c r="H4" s="1" t="n"/>
       <c r="I4" s="9" t="n">
         <v>620</v>
@@ -1052,9 +1074,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E5" s="1" t="n"/>
-      <c r="F5" s="1" t="n"/>
-      <c r="G5" s="46" t="n"/>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" s="46" t="inlineStr">
+        <is>
+          <t>BTICINO</t>
+        </is>
+      </c>
       <c r="H5" s="1" t="n"/>
       <c r="I5" s="8" t="n">
         <v>766</v>
@@ -1090,9 +1122,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E6" s="1" t="n"/>
-      <c r="F6" s="1" t="n"/>
-      <c r="G6" s="46" t="n"/>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" s="46" t="inlineStr">
+        <is>
+          <t>BTICINO</t>
+        </is>
+      </c>
       <c r="H6" s="1" t="n"/>
       <c r="I6" s="8" t="n">
         <v>1158</v>
@@ -1129,9 +1171,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E7" s="1" t="n"/>
-      <c r="F7" s="1" t="n"/>
-      <c r="G7" s="46" t="n"/>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G7" s="46" t="inlineStr">
+        <is>
+          <t>BTICINO</t>
+        </is>
+      </c>
       <c r="H7" s="1" t="n"/>
       <c r="I7" s="8" t="n">
         <v>1664</v>
@@ -1168,9 +1220,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E8" s="1" t="n"/>
-      <c r="F8" s="1" t="n"/>
-      <c r="G8" s="46" t="n"/>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G8" s="46" t="inlineStr">
+        <is>
+          <t>BTICINO</t>
+        </is>
+      </c>
       <c r="H8" s="1" t="n"/>
       <c r="I8" s="8" t="n">
         <v>857</v>
@@ -1207,9 +1269,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E9" s="1" t="n"/>
-      <c r="F9" s="1" t="n"/>
-      <c r="G9" s="46" t="n"/>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G9" s="46" t="inlineStr">
+        <is>
+          <t>BTICINO</t>
+        </is>
+      </c>
       <c r="H9" s="1" t="n"/>
       <c r="I9" s="8" t="n">
         <v>1272</v>
@@ -1245,9 +1317,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E10" s="1" t="n"/>
-      <c r="F10" s="1" t="n"/>
-      <c r="G10" s="46" t="n"/>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G10" s="46" t="inlineStr">
+        <is>
+          <t>BTICINO</t>
+        </is>
+      </c>
       <c r="H10" s="1" t="n"/>
       <c r="I10" s="8" t="n">
         <v>1550</v>
@@ -1283,8 +1365,14 @@
           <t>PAQUETE</t>
         </is>
       </c>
-      <c r="E11" s="1" t="n"/>
-      <c r="F11" s="1" t="n"/>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G11" s="46" t="n"/>
       <c r="H11" s="1" t="n"/>
       <c r="I11" s="8" t="n">
@@ -1319,8 +1407,14 @@
           <t>PAQUETE</t>
         </is>
       </c>
-      <c r="E12" s="1" t="n"/>
-      <c r="F12" s="1" t="n"/>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G12" s="46" t="n"/>
       <c r="H12" s="1" t="n"/>
       <c r="I12" s="8" t="n">
@@ -1355,9 +1449,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E13" s="1" t="n"/>
-      <c r="F13" s="1" t="n"/>
-      <c r="G13" s="46" t="n"/>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G13" s="46" t="inlineStr">
+        <is>
+          <t>PHILCO</t>
+        </is>
+      </c>
       <c r="H13" s="1" t="n"/>
       <c r="I13" s="8" t="n">
         <v>40</v>
@@ -1393,8 +1497,14 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E14" s="1" t="n"/>
-      <c r="F14" s="1" t="n"/>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G14" s="46" t="n"/>
       <c r="H14" s="1" t="n"/>
       <c r="I14" s="8" t="n">
@@ -1431,8 +1541,14 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E15" s="1" t="n"/>
-      <c r="F15" s="1" t="n"/>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G15" s="46" t="inlineStr">
         <is>
           <t>THORSMAN</t>
@@ -1471,9 +1587,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E16" s="1" t="n"/>
-      <c r="F16" s="1" t="n"/>
-      <c r="G16" s="46" t="n"/>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G16" s="46" t="inlineStr">
+        <is>
+          <t>SQUARE D</t>
+        </is>
+      </c>
       <c r="H16" s="1" t="n"/>
       <c r="I16" s="8" t="n">
         <v>195.4</v>
@@ -1507,9 +1633,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E17" s="1" t="n"/>
-      <c r="F17" s="1" t="n"/>
-      <c r="G17" s="46" t="n"/>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G17" s="46" t="inlineStr">
+        <is>
+          <t>SQUARE D</t>
+        </is>
+      </c>
       <c r="H17" s="1" t="n"/>
       <c r="I17" s="10" t="n">
         <v>382</v>
@@ -1543,9 +1679,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E18" s="1" t="n"/>
-      <c r="F18" s="1" t="n"/>
-      <c r="G18" s="46" t="n"/>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G18" s="46" t="inlineStr">
+        <is>
+          <t>NACIONAL</t>
+        </is>
+      </c>
       <c r="H18" s="1" t="n"/>
       <c r="I18" s="10" t="n">
         <v>129.6</v>
@@ -1579,9 +1725,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E19" s="1" t="n"/>
-      <c r="F19" s="1" t="n"/>
-      <c r="G19" s="46" t="n"/>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G19" s="46" t="inlineStr">
+        <is>
+          <t>3M</t>
+        </is>
+      </c>
       <c r="H19" s="1" t="n"/>
       <c r="I19" s="10" t="n">
         <v>86</v>
@@ -1615,9 +1771,19 @@
           <t>JUEGO</t>
         </is>
       </c>
-      <c r="E20" s="1" t="n"/>
-      <c r="F20" s="1" t="n"/>
-      <c r="G20" s="46" t="n"/>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>ESTADOS UNIDOS</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="G20" s="46" t="inlineStr">
+        <is>
+          <t>nVENT ERICO</t>
+        </is>
+      </c>
       <c r="H20" s="1" t="n"/>
       <c r="I20" s="11" t="n"/>
       <c r="J20" s="8" t="n"/>
@@ -1642,9 +1808,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E21" s="1" t="n"/>
-      <c r="F21" s="1" t="n"/>
-      <c r="G21" s="46" t="n"/>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G21" s="46" t="inlineStr">
+        <is>
+          <t>BTICINO</t>
+        </is>
+      </c>
       <c r="H21" s="1" t="n"/>
       <c r="I21" s="10" t="n">
         <v>89</v>
@@ -1678,9 +1854,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E22" s="1" t="n"/>
-      <c r="F22" s="1" t="n"/>
-      <c r="G22" s="46" t="n"/>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G22" s="46" t="inlineStr">
+        <is>
+          <t>BTICINO</t>
+        </is>
+      </c>
       <c r="H22" s="1" t="n"/>
       <c r="I22" s="10" t="n">
         <v>280</v>
@@ -1714,9 +1900,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E23" s="1" t="n"/>
-      <c r="F23" s="1" t="n"/>
-      <c r="G23" s="46" t="n"/>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G23" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H23" s="1" t="n"/>
       <c r="I23" s="10" t="n">
         <v>120</v>
@@ -1752,9 +1948,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E24" s="1" t="n"/>
-      <c r="F24" s="1" t="n"/>
-      <c r="G24" s="46" t="n"/>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G24" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H24" s="1" t="n"/>
       <c r="I24" s="10" t="n">
         <v>26</v>
@@ -1790,9 +1996,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E25" s="1" t="n"/>
-      <c r="F25" s="1" t="n"/>
-      <c r="G25" s="46" t="n"/>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G25" s="46" t="inlineStr">
+        <is>
+          <t>SQUARE D</t>
+        </is>
+      </c>
       <c r="H25" s="1" t="n"/>
       <c r="I25" s="10" t="n">
         <v>437</v>
@@ -1826,9 +2042,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E26" s="1" t="n"/>
-      <c r="F26" s="1" t="n"/>
-      <c r="G26" s="46" t="n"/>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G26" s="46" t="inlineStr">
+        <is>
+          <t>SQUARE D</t>
+        </is>
+      </c>
       <c r="H26" s="1" t="n"/>
       <c r="I26" s="10" t="n">
         <v>437</v>
@@ -1862,9 +2088,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E27" s="1" t="n"/>
-      <c r="F27" s="1" t="n"/>
-      <c r="G27" s="46" t="n"/>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G27" s="46" t="inlineStr">
+        <is>
+          <t>SQUARE D</t>
+        </is>
+      </c>
       <c r="H27" s="47" t="n"/>
       <c r="I27" s="55" t="n">
         <v>1023</v>
@@ -1898,9 +2134,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E28" s="1" t="n"/>
-      <c r="F28" s="1" t="n"/>
-      <c r="G28" s="47" t="n"/>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G28" s="47" t="inlineStr">
+        <is>
+          <t>SQUARE D</t>
+        </is>
+      </c>
       <c r="H28" s="46" t="n"/>
       <c r="I28" s="57" t="n">
         <v>3068</v>
@@ -1934,9 +2180,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E29" s="1" t="n"/>
-      <c r="F29" s="1" t="n"/>
-      <c r="G29" s="46" t="n"/>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G29" s="46" t="inlineStr">
+        <is>
+          <t>SQUARE D</t>
+        </is>
+      </c>
       <c r="H29" s="46" t="n"/>
       <c r="I29" s="57" t="n"/>
       <c r="J29" s="57" t="n"/>
@@ -1961,9 +2217,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E30" s="1" t="n"/>
-      <c r="F30" s="1" t="n"/>
-      <c r="G30" s="46" t="n"/>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G30" s="46" t="inlineStr">
+        <is>
+          <t>SQUARE D</t>
+        </is>
+      </c>
       <c r="H30" s="53" t="n"/>
       <c r="I30" s="10" t="n">
         <v>1681</v>
@@ -1997,9 +2263,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E31" s="1" t="n"/>
-      <c r="F31" s="1" t="n"/>
-      <c r="G31" s="46" t="n"/>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G31" s="46" t="inlineStr">
+        <is>
+          <t>SQUARE D</t>
+        </is>
+      </c>
       <c r="H31" s="1" t="n"/>
       <c r="I31" s="10" t="n">
         <v>1681</v>
@@ -2033,9 +2309,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E32" s="1" t="n"/>
-      <c r="F32" s="1" t="n"/>
-      <c r="G32" s="46" t="n"/>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G32" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H32" s="1" t="n"/>
       <c r="I32" s="10" t="n">
         <v>1681</v>
@@ -2069,9 +2355,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E33" s="1" t="n"/>
-      <c r="F33" s="1" t="n"/>
-      <c r="G33" s="46" t="n"/>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G33" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H33" s="1" t="n"/>
       <c r="I33" s="10" t="n">
         <v>990</v>
@@ -2107,9 +2403,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E34" s="1" t="n"/>
-      <c r="F34" s="1" t="n"/>
-      <c r="G34" s="46" t="n"/>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G34" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H34" s="1" t="n"/>
       <c r="I34" s="10" t="n">
         <v>938</v>
@@ -2145,9 +2451,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E35" s="1" t="n"/>
-      <c r="F35" s="1" t="n"/>
-      <c r="G35" s="46" t="n"/>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G35" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H35" s="1" t="n"/>
       <c r="I35" s="10" t="n">
         <v>101</v>
@@ -2181,9 +2497,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E36" s="1" t="n"/>
-      <c r="F36" s="1" t="n"/>
-      <c r="G36" s="46" t="n"/>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G36" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H36" s="1" t="n"/>
       <c r="I36" s="10" t="n">
         <v>101</v>
@@ -2217,9 +2543,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E37" s="1" t="n"/>
-      <c r="F37" s="1" t="n"/>
-      <c r="G37" s="46" t="n"/>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G37" s="46" t="inlineStr">
+        <is>
+          <t>PHILCO</t>
+        </is>
+      </c>
       <c r="H37" s="1" t="n"/>
       <c r="I37" s="10" t="n">
         <v>380</v>
@@ -2255,9 +2591,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E38" s="1" t="n"/>
-      <c r="F38" s="1" t="n"/>
-      <c r="G38" s="46" t="n"/>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G38" s="46" t="inlineStr">
+        <is>
+          <t>PHILCO</t>
+        </is>
+      </c>
       <c r="H38" s="1" t="n"/>
       <c r="I38" s="10" t="n">
         <v>380</v>
@@ -2294,9 +2640,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E39" s="1" t="n"/>
-      <c r="F39" s="1" t="n"/>
-      <c r="G39" s="46" t="n"/>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F39" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G39" s="46" t="inlineStr">
+        <is>
+          <t>PHILCO</t>
+        </is>
+      </c>
       <c r="H39" s="1" t="n"/>
       <c r="I39" s="10" t="n">
         <v>615</v>
@@ -2333,9 +2689,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E40" s="1" t="n"/>
-      <c r="F40" s="1" t="n"/>
-      <c r="G40" s="46" t="n"/>
+      <c r="E40" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F40" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G40" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H40" s="1" t="n"/>
       <c r="I40" s="10" t="n">
         <v>790</v>
@@ -2372,9 +2738,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E41" s="1" t="n"/>
-      <c r="F41" s="1" t="n"/>
-      <c r="G41" s="46" t="n"/>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F41" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G41" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H41" s="1" t="n"/>
       <c r="I41" s="10" t="n">
         <v>690</v>
@@ -2408,9 +2784,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E42" s="1" t="n"/>
-      <c r="F42" s="1" t="n"/>
-      <c r="G42" s="46" t="n"/>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F42" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G42" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H42" s="1" t="n"/>
       <c r="I42" s="10" t="n">
         <v>83</v>
@@ -2446,9 +2832,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E43" s="1" t="n"/>
-      <c r="F43" s="1" t="n"/>
-      <c r="G43" s="46" t="n"/>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G43" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H43" s="1" t="n"/>
       <c r="I43" s="10" t="n">
         <v>148</v>
@@ -2482,8 +2878,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E44" s="1" t="n"/>
-      <c r="F44" s="1" t="n"/>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H44" s="1" t="n"/>
       <c r="I44" s="10" t="n">
         <v>148</v>
@@ -2516,8 +2923,14 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E45" s="1" t="n"/>
-      <c r="F45" s="1" t="n"/>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>ESTADOS UNIDOS</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G45" s="46" t="inlineStr">
         <is>
           <t>KLEIN TOOLS</t>
@@ -2556,8 +2969,14 @@
           <t>PAQUETE</t>
         </is>
       </c>
-      <c r="E46" s="1" t="n"/>
-      <c r="F46" s="1" t="n"/>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F46" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G46" s="46" t="inlineStr">
         <is>
           <t>SURTEK</t>
@@ -2596,8 +3015,14 @@
           <t>PAQUETE</t>
         </is>
       </c>
-      <c r="E47" s="1" t="n"/>
-      <c r="F47" s="1" t="n"/>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G47" s="46" t="inlineStr">
         <is>
           <t>SURTEK</t>
@@ -2636,8 +3061,14 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E48" s="1" t="n"/>
-      <c r="F48" s="1" t="n"/>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G48" s="46" t="inlineStr">
         <is>
           <t>STEREN</t>
@@ -2676,8 +3107,14 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E49" s="1" t="n"/>
-      <c r="F49" s="1" t="n"/>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G49" s="46" t="inlineStr">
         <is>
           <t>SURTEK</t>
@@ -2716,8 +3153,14 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E50" s="1" t="n"/>
-      <c r="F50" s="1" t="n"/>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>ESTADOS UNIDOS</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G50" s="46" t="inlineStr">
         <is>
           <t>KLEIN TOOLS</t>
@@ -2756,8 +3199,14 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E51" s="1" t="n"/>
-      <c r="F51" s="1" t="n"/>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G51" s="46" t="inlineStr">
         <is>
           <t>SURTEK</t>
@@ -2796,9 +3245,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E52" s="1" t="n"/>
-      <c r="F52" s="1" t="n"/>
-      <c r="G52" s="46" t="n"/>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F52" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G52" s="46" t="inlineStr">
+        <is>
+          <t>BTICINO</t>
+        </is>
+      </c>
       <c r="H52" s="1" t="n"/>
       <c r="I52" s="10" t="n">
         <v>119</v>
@@ -2832,9 +3291,19 @@
           <t>CAJA</t>
         </is>
       </c>
-      <c r="E53" s="1" t="n"/>
-      <c r="F53" s="1" t="n"/>
-      <c r="G53" s="46" t="n"/>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G53" s="46" t="inlineStr">
+        <is>
+          <t>BTICINO</t>
+        </is>
+      </c>
       <c r="H53" s="1" t="n"/>
       <c r="I53" s="10" t="n">
         <v>181</v>
@@ -2868,8 +3337,14 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E54" s="1" t="n"/>
-      <c r="F54" s="1" t="n"/>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G54" s="46" t="inlineStr">
         <is>
           <t>ESTEVEZ</t>
@@ -2908,8 +3383,14 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E55" s="1" t="n"/>
-      <c r="F55" s="1" t="n"/>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F55" s="1" t="n">
+        <v>100</v>
+      </c>
       <c r="G55" s="46" t="n"/>
       <c r="H55" s="1" t="n"/>
       <c r="I55" s="10" t="n">
@@ -2946,9 +3427,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E56" s="1" t="n"/>
-      <c r="F56" s="1" t="n"/>
-      <c r="G56" s="46" t="n"/>
+      <c r="E56" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F56" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G56" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H56" s="1" t="n"/>
       <c r="I56" s="10" t="n">
         <v>237.9</v>
@@ -2982,9 +3473,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E57" s="1" t="n"/>
-      <c r="F57" s="1" t="n"/>
-      <c r="G57" s="46" t="n"/>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F57" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G57" s="46" t="inlineStr">
+        <is>
+          <t>PHILCO</t>
+        </is>
+      </c>
       <c r="H57" s="1" t="n"/>
       <c r="I57" s="10" t="n">
         <v>1420</v>
@@ -3020,9 +3521,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E58" s="1" t="n"/>
-      <c r="F58" s="1" t="n"/>
-      <c r="G58" s="46" t="n"/>
+      <c r="E58" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F58" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G58" s="46" t="inlineStr">
+        <is>
+          <t>PHILCO</t>
+        </is>
+      </c>
       <c r="H58" s="1" t="n"/>
       <c r="I58" s="10" t="n">
         <v>189</v>
@@ -3058,9 +3569,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E59" s="1" t="n"/>
-      <c r="F59" s="1" t="n"/>
-      <c r="G59" s="46" t="n"/>
+      <c r="E59" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F59" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G59" s="46" t="inlineStr">
+        <is>
+          <t>PHILCO</t>
+        </is>
+      </c>
       <c r="H59" s="1" t="n"/>
       <c r="I59" s="10" t="n">
         <v>277</v>
@@ -3096,9 +3617,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E60" s="1" t="n"/>
-      <c r="F60" s="1" t="n"/>
-      <c r="G60" s="46" t="n"/>
+      <c r="E60" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F60" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G60" s="46" t="inlineStr">
+        <is>
+          <t>PHILCO</t>
+        </is>
+      </c>
       <c r="H60" s="1" t="n"/>
       <c r="I60" s="10" t="n">
         <v>630</v>
@@ -3134,9 +3665,19 @@
           <t>ROLLO</t>
         </is>
       </c>
-      <c r="E61" s="1" t="n"/>
-      <c r="F61" s="1" t="n"/>
-      <c r="G61" s="46" t="n"/>
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F61" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G61" s="46" t="inlineStr">
+        <is>
+          <t>CONDUMEX</t>
+        </is>
+      </c>
       <c r="H61" s="1" t="n"/>
       <c r="I61" s="10" t="n"/>
       <c r="J61" s="60" t="n">
@@ -3170,9 +3711,19 @@
           <t>ROLLO</t>
         </is>
       </c>
-      <c r="E62" s="1" t="n"/>
-      <c r="F62" s="1" t="n"/>
-      <c r="G62" s="46" t="n"/>
+      <c r="E62" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F62" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G62" s="46" t="inlineStr">
+        <is>
+          <t>CONDUMEX</t>
+        </is>
+      </c>
       <c r="H62" s="1" t="n"/>
       <c r="I62" s="10" t="n">
         <v>4740</v>
@@ -3206,9 +3757,19 @@
           <t>ROLLO</t>
         </is>
       </c>
-      <c r="E63" s="1" t="n"/>
-      <c r="F63" s="1" t="n"/>
-      <c r="G63" s="46" t="n"/>
+      <c r="E63" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F63" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G63" s="46" t="inlineStr">
+        <is>
+          <t>CONDUMEX</t>
+        </is>
+      </c>
       <c r="H63" s="1" t="n"/>
       <c r="I63" s="10" t="n">
         <v>2990</v>
@@ -3242,9 +3803,19 @@
           <t>ROLLO</t>
         </is>
       </c>
-      <c r="E64" s="1" t="n"/>
-      <c r="F64" s="1" t="n"/>
-      <c r="G64" s="46" t="n"/>
+      <c r="E64" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F64" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G64" s="46" t="inlineStr">
+        <is>
+          <t>CONDUMEX</t>
+        </is>
+      </c>
       <c r="H64" s="1" t="n"/>
       <c r="I64" s="10" t="n">
         <v>1850</v>
@@ -3278,9 +3849,19 @@
           <t>ROLLO</t>
         </is>
       </c>
-      <c r="E65" s="1" t="n"/>
-      <c r="F65" s="1" t="n"/>
-      <c r="G65" s="46" t="n"/>
+      <c r="E65" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F65" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G65" s="46" t="inlineStr">
+        <is>
+          <t>CONDUMEX</t>
+        </is>
+      </c>
       <c r="H65" s="1" t="n"/>
       <c r="I65" s="10" t="n">
         <v>1190</v>
@@ -3314,9 +3895,19 @@
           <t>ROLLO</t>
         </is>
       </c>
-      <c r="E66" s="1" t="n"/>
-      <c r="F66" s="1" t="n"/>
-      <c r="G66" s="46" t="n"/>
+      <c r="E66" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F66" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G66" s="46" t="inlineStr">
+        <is>
+          <t>CONDUMEX</t>
+        </is>
+      </c>
       <c r="H66" s="1" t="n"/>
       <c r="I66" s="10" t="n">
         <v>840</v>
@@ -3350,9 +3941,19 @@
           <t>ROLLO</t>
         </is>
       </c>
-      <c r="E67" s="1" t="n"/>
-      <c r="F67" s="1" t="n"/>
-      <c r="G67" s="46" t="n"/>
+      <c r="E67" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F67" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G67" s="46" t="inlineStr">
+        <is>
+          <t>CONDUMEX</t>
+        </is>
+      </c>
       <c r="H67" s="1" t="n"/>
       <c r="I67" s="10" t="n">
         <v>620</v>
@@ -3386,9 +3987,19 @@
           <t>ROLLO</t>
         </is>
       </c>
-      <c r="E68" s="1" t="n"/>
-      <c r="F68" s="1" t="n"/>
-      <c r="G68" s="46" t="n"/>
+      <c r="E68" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F68" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G68" s="46" t="inlineStr">
+        <is>
+          <t>CONDUMEX</t>
+        </is>
+      </c>
       <c r="H68" s="1" t="n"/>
       <c r="I68" s="10" t="n">
         <v>3540</v>
@@ -3422,9 +4033,19 @@
           <t>ROLLO</t>
         </is>
       </c>
-      <c r="E69" s="1" t="n"/>
-      <c r="F69" s="1" t="n"/>
-      <c r="G69" s="46" t="n"/>
+      <c r="E69" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F69" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G69" s="46" t="inlineStr">
+        <is>
+          <t>CONDUMEX</t>
+        </is>
+      </c>
       <c r="H69" s="1" t="n"/>
       <c r="I69" s="10" t="n">
         <v>2480</v>
@@ -3458,9 +4079,19 @@
           <t>ROLLO</t>
         </is>
       </c>
-      <c r="E70" s="1" t="n"/>
-      <c r="F70" s="1" t="n"/>
-      <c r="G70" s="46" t="n"/>
+      <c r="E70" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F70" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G70" s="46" t="inlineStr">
+        <is>
+          <t>CONDUMEX</t>
+        </is>
+      </c>
       <c r="H70" s="1" t="n"/>
       <c r="I70" s="10" t="n">
         <v>2220</v>
@@ -3494,9 +4125,19 @@
           <t>ROLLO</t>
         </is>
       </c>
-      <c r="E71" s="1" t="n"/>
-      <c r="F71" s="1" t="n"/>
-      <c r="G71" s="46" t="n"/>
+      <c r="E71" s="1" t="inlineStr">
+        <is>
+          <t>MEXICO</t>
+        </is>
+      </c>
+      <c r="F71" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G71" s="46" t="inlineStr">
+        <is>
+          <t>CONDUMEX</t>
+        </is>
+      </c>
       <c r="H71" s="1" t="n"/>
       <c r="I71" s="10" t="n">
         <v>2620</v>
@@ -3530,9 +4171,19 @@
           <t>PIEZA</t>
         </is>
       </c>
-      <c r="E72" s="1" t="n"/>
-      <c r="F72" s="1" t="n"/>
-      <c r="G72" s="52" t="n"/>
+      <c r="E72" s="1" t="inlineStr">
+        <is>
+          <t>CHINA</t>
+        </is>
+      </c>
+      <c r="F72" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="52" t="inlineStr">
+        <is>
+          <t>NACIONAL</t>
+        </is>
+      </c>
       <c r="H72" s="1" t="n"/>
       <c r="I72" s="10" t="n">
         <v>1740</v>

</xml_diff>

<commit_message>
Complete columns E, F, G (país, integración, marca) for all sheet 1 items
Co-authored-by: Miguel Angel Cruz Ortiz <Ylika.dev@outlook.com>
</commit_message>
<xml_diff>
--- a/ANEXO TECNICO POLICIA BANCARIA.xlsx
+++ b/ANEXO TECNICO POLICIA BANCARIA.xlsx
@@ -952,7 +952,11 @@
       <c r="F2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="46" t="n"/>
+      <c r="G2" s="46" t="inlineStr">
+        <is>
+          <t>NACIONAL</t>
+        </is>
+      </c>
       <c r="H2" s="1" t="n"/>
       <c r="I2" s="8" t="n"/>
       <c r="J2" s="14" t="n"/>
@@ -994,7 +998,11 @@
       <c r="F3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="46" t="n"/>
+      <c r="G3" s="46" t="inlineStr">
+        <is>
+          <t>NACIONAL</t>
+        </is>
+      </c>
       <c r="H3" s="1" t="n"/>
       <c r="I3" s="8" t="n"/>
       <c r="J3" s="14" t="n"/>
@@ -1373,7 +1381,11 @@
       <c r="F11" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G11" s="46" t="n"/>
+      <c r="G11" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H11" s="1" t="n"/>
       <c r="I11" s="8" t="n">
         <v>350</v>
@@ -1415,7 +1427,11 @@
       <c r="F12" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G12" s="46" t="n"/>
+      <c r="G12" s="46" t="inlineStr">
+        <is>
+          <t>PEFSA</t>
+        </is>
+      </c>
       <c r="H12" s="1" t="n"/>
       <c r="I12" s="8" t="n">
         <v>310</v>
@@ -1505,7 +1521,11 @@
       <c r="F14" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G14" s="46" t="n"/>
+      <c r="G14" s="46" t="inlineStr">
+        <is>
+          <t>FONTANA</t>
+        </is>
+      </c>
       <c r="H14" s="1" t="n"/>
       <c r="I14" s="8" t="n">
         <v>68.59999999999999</v>
@@ -3391,7 +3411,11 @@
       <c r="F55" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G55" s="46" t="n"/>
+      <c r="G55" s="46" t="inlineStr">
+        <is>
+          <t>ESTEVEZ</t>
+        </is>
+      </c>
       <c r="H55" s="1" t="n"/>
       <c r="I55" s="10" t="n">
         <v>183.5</v>

</xml_diff>

<commit_message>
Fix origin logic: Philco and LED imports as CHINA 0%, keep Mexican-made products
Co-authored-by: Miguel Angel Cruz Ortiz <Ylika.dev@outlook.com>
</commit_message>
<xml_diff>
--- a/ANEXO TECNICO POLICIA BANCARIA.xlsx
+++ b/ANEXO TECNICO POLICIA BANCARIA.xlsx
@@ -1375,11 +1375,11 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F11" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G11" s="46" t="inlineStr">
         <is>
@@ -1421,11 +1421,11 @@
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F12" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G12" s="46" t="inlineStr">
         <is>
@@ -1467,11 +1467,11 @@
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F13" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G13" s="46" t="inlineStr">
         <is>
@@ -1922,11 +1922,11 @@
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F23" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G23" s="46" t="inlineStr">
         <is>
@@ -1970,11 +1970,11 @@
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F24" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G24" s="46" t="inlineStr">
         <is>
@@ -2331,11 +2331,11 @@
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F32" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G32" s="46" t="inlineStr">
         <is>
@@ -2377,11 +2377,11 @@
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F33" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G33" s="46" t="inlineStr">
         <is>
@@ -2425,11 +2425,11 @@
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F34" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G34" s="46" t="inlineStr">
         <is>
@@ -2473,11 +2473,11 @@
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F35" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G35" s="46" t="inlineStr">
         <is>
@@ -2519,11 +2519,11 @@
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F36" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G36" s="46" t="inlineStr">
         <is>
@@ -2565,11 +2565,11 @@
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F37" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G37" s="46" t="inlineStr">
         <is>
@@ -2613,11 +2613,11 @@
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F38" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G38" s="46" t="inlineStr">
         <is>
@@ -2662,11 +2662,11 @@
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F39" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G39" s="46" t="inlineStr">
         <is>
@@ -2711,11 +2711,11 @@
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F40" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G40" s="46" t="inlineStr">
         <is>
@@ -2760,11 +2760,11 @@
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F41" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G41" s="46" t="inlineStr">
         <is>
@@ -2806,11 +2806,11 @@
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F42" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G42" s="46" t="inlineStr">
         <is>
@@ -2854,11 +2854,11 @@
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F43" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G43" s="46" t="inlineStr">
         <is>
@@ -2900,11 +2900,11 @@
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F44" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -3453,11 +3453,11 @@
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F56" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G56" s="46" t="inlineStr">
         <is>
@@ -3499,11 +3499,11 @@
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F57" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G57" s="46" t="inlineStr">
         <is>
@@ -3547,11 +3547,11 @@
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F58" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G58" s="46" t="inlineStr">
         <is>
@@ -3595,11 +3595,11 @@
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F59" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G59" s="46" t="inlineStr">
         <is>
@@ -3643,11 +3643,11 @@
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F60" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G60" s="46" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Set sheet 1 origin by actual manufacturing country, not distributor
Co-authored-by: Miguel Angel Cruz Ortiz <Ylika.dev@outlook.com>
</commit_message>
<xml_diff>
--- a/ANEXO TECNICO POLICIA BANCARIA.xlsx
+++ b/ANEXO TECNICO POLICIA BANCARIA.xlsx
@@ -1383,7 +1383,7 @@
       </c>
       <c r="G11" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H11" s="1" t="n"/>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G12" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H12" s="1" t="n"/>
@@ -1830,15 +1830,15 @@
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F21" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G21" s="46" t="inlineStr">
         <is>
-          <t>BTICINO</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H21" s="1" t="n"/>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="G23" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H23" s="1" t="n"/>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="G24" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H24" s="1" t="n"/>
@@ -2339,7 +2339,7 @@
       </c>
       <c r="G32" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H32" s="1" t="n"/>
@@ -2385,7 +2385,7 @@
       </c>
       <c r="G33" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H33" s="1" t="n"/>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="G34" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H34" s="1" t="n"/>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="G35" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H35" s="1" t="n"/>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="G36" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H36" s="1" t="n"/>
@@ -2719,7 +2719,7 @@
       </c>
       <c r="G40" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H40" s="1" t="n"/>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="G41" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H41" s="1" t="n"/>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="G42" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H42" s="1" t="n"/>
@@ -2862,7 +2862,7 @@
       </c>
       <c r="G43" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H43" s="1" t="n"/>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H44" s="1" t="n"/>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>ESTADOS UNIDOS</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F45" s="1" t="n">
@@ -2991,11 +2991,11 @@
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F46" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G46" s="46" t="inlineStr">
         <is>
@@ -3037,11 +3037,11 @@
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F47" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G47" s="46" t="inlineStr">
         <is>
@@ -3083,11 +3083,11 @@
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F48" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G48" s="46" t="inlineStr">
         <is>
@@ -3129,11 +3129,11 @@
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F49" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G49" s="46" t="inlineStr">
         <is>
@@ -3175,7 +3175,7 @@
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>ESTADOS UNIDOS</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F50" s="1" t="n">
@@ -3221,11 +3221,11 @@
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F51" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G51" s="46" t="inlineStr">
         <is>
@@ -3405,15 +3405,15 @@
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>MEXICO</t>
+          <t>CHINA</t>
         </is>
       </c>
       <c r="F55" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G55" s="46" t="inlineStr">
         <is>
-          <t>ESTEVEZ</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H55" s="1" t="n"/>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="G56" s="46" t="inlineStr">
         <is>
-          <t>PEFSA</t>
+          <t>NACIONAL</t>
         </is>
       </c>
       <c r="H56" s="1" t="n"/>

</xml_diff>